<commit_message>
test(xlsx-agent): sync Blixt fixture + assert sponsor_name populate
</commit_message>
<xml_diff>
--- a/apps/agents/xlsx-agent/tests/fixtures/blixt-lbo-v1.xlsx
+++ b/apps/agents/xlsx-agent/tests/fixtures/blixt-lbo-v1.xlsx
@@ -7764,7 +7764,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="en-US"/>
               </a:p>
@@ -8932,7 +8932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A8:J48"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="3.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -9145,7 +9145,13 @@
     <row r="9" ht="15" customFormat="1" customHeight="1" s="149">
       <c r="A9" s="165" t="n"/>
     </row>
-    <row r="10" ht="15" customHeight="1"/>
+    <row r="10" ht="15" customHeight="1">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Blixt</t>
+        </is>
+      </c>
+    </row>
     <row r="11" ht="15" customHeight="1">
       <c r="B11" s="1035">
         <f>NOW()</f>
@@ -35525,7 +35531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B3:I8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.5703125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -35535,6 +35541,8 @@
     <col width="18.28515625" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3">
       <c r="C3" s="772" t="n">
         <v>45658</v>
@@ -35638,6 +35646,7 @@
         <v/>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
@@ -35739,10 +35748,9 @@
         <f>Cover!$B$8</f>
         <v/>
       </c>
-      <c r="I3" s="387" t="inlineStr">
-        <is>
-          <t>Blixt returns summary</t>
-        </is>
+      <c r="I3" s="387">
+        <f>Cover!$B$10&amp;" returns summary"</f>
+        <v/>
       </c>
       <c r="J3" s="121" t="n"/>
       <c r="K3" s="1045">
@@ -36269,10 +36277,9 @@
         <f>+G17*F20</f>
         <v/>
       </c>
-      <c r="I20" s="1" t="inlineStr">
-        <is>
-          <t>Blixt exit fee (% EV)</t>
-        </is>
+      <c r="I20" s="1">
+        <f>Cover!$B$10&amp;" exit fee (% EV)"</f>
+        <v/>
       </c>
       <c r="L20" s="1067" t="n"/>
       <c r="U20" s="617" t="inlineStr">
@@ -36332,10 +36339,9 @@
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="307" t="n"/>
-      <c r="B24" s="1" t="inlineStr">
-        <is>
-          <t>Blixt preferred equity</t>
-        </is>
+      <c r="B24" s="1">
+        <f>Cover!$B$10&amp;" preferred equity"</f>
+        <v/>
       </c>
       <c r="G24" s="1067" t="n"/>
       <c r="I24" s="1" t="inlineStr">
@@ -38256,10 +38262,9 @@
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="307" t="n"/>
-      <c r="B66" s="1" t="inlineStr">
-        <is>
-          <t>Blixt (Day 1)</t>
-        </is>
+      <c r="B66" s="1">
+        <f>Cover!$B$10&amp;" (Day 1)"</f>
+        <v/>
       </c>
       <c r="D66" s="353" t="n"/>
       <c r="E66" s="353" t="n"/>
@@ -38705,10 +38710,9 @@
       <c r="P70" s="658" t="n"/>
       <c r="Q70" s="1151" t="n"/>
       <c r="R70" s="1150" t="n"/>
-      <c r="U70" s="419" t="inlineStr">
-        <is>
-          <t>Blixt injections</t>
-        </is>
+      <c r="U70" s="419">
+        <f>Cover!$B$10&amp;" injections"</f>
+        <v/>
       </c>
       <c r="V70" s="420" t="n"/>
       <c r="W70" s="420" t="n"/>
@@ -39091,10 +39095,9 @@
       <c r="P77" s="1150" t="n"/>
       <c r="Q77" s="1150" t="n"/>
       <c r="R77" s="1150" t="n"/>
-      <c r="U77" s="20" t="inlineStr">
-        <is>
-          <t>Blixt</t>
-        </is>
+      <c r="U77" s="20">
+        <f>Cover!$B$10</f>
+        <v/>
       </c>
       <c r="V77" s="5" t="n"/>
       <c r="W77" s="5" t="n"/>
@@ -39392,10 +39395,9 @@
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="307" t="n"/>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>Blixt loan note / prior ranking</t>
-        </is>
+      <c r="B83" s="2">
+        <f>Cover!$B$10&amp;" loan note / prior ranking"</f>
+        <v/>
       </c>
       <c r="E83" s="1173">
         <f>+N66</f>
@@ -39469,10 +39471,9 @@
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="307" t="n"/>
-      <c r="B85" s="24" t="inlineStr">
-        <is>
-          <t>Blixt</t>
-        </is>
+      <c r="B85" s="24">
+        <f>Cover!$B$10</f>
+        <v/>
       </c>
       <c r="D85" s="367">
         <f>+E85/$E$89</f>
@@ -39736,10 +39737,9 @@
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" s="307" t="n"/>
-      <c r="B91" s="24" t="inlineStr">
-        <is>
-          <t>Blixt</t>
-        </is>
+      <c r="B91" s="24">
+        <f>Cover!$B$10</f>
+        <v/>
       </c>
       <c r="D91" s="367">
         <f>+E91/$E$95</f>
@@ -40128,10 +40128,9 @@
     </row>
     <row r="102" outlineLevel="1" ht="15" customHeight="1">
       <c r="A102" s="307" t="n"/>
-      <c r="B102" s="72" t="inlineStr">
-        <is>
-          <t>Total Blixt Equity</t>
-        </is>
+      <c r="B102" s="72">
+        <f>"Total "&amp;Cover!$B$10&amp;" Equity"</f>
+        <v/>
       </c>
       <c r="E102" s="1062">
         <f>+E91+E85</f>
@@ -45020,10 +45019,9 @@
     </row>
     <row r="218" ht="15" customHeight="1">
       <c r="A218" s="307" t="n"/>
-      <c r="B218" s="1" t="inlineStr">
-        <is>
-          <t>Blixt management fee</t>
-        </is>
+      <c r="B218" s="1">
+        <f>Cover!$B$10&amp;" management fee"</f>
+        <v/>
       </c>
       <c r="E218" s="353" t="n"/>
       <c r="F218" s="353" t="n"/>
@@ -45471,10 +45469,9 @@
     </row>
     <row r="231" ht="15" customFormat="1" customHeight="1" s="21">
       <c r="A231" s="459" t="n"/>
-      <c r="B231" s="1" t="inlineStr">
-        <is>
-          <t>Blixt new equity</t>
-        </is>
+      <c r="B231" s="1">
+        <f>Cover!$B$10&amp;" new equity"</f>
+        <v/>
       </c>
       <c r="C231" s="7" t="n"/>
       <c r="D231" s="7" t="n"/>
@@ -47352,10 +47349,9 @@
     </row>
     <row r="297" ht="15" customHeight="1">
       <c r="A297" s="307" t="n"/>
-      <c r="B297" s="306" t="inlineStr">
-        <is>
-          <t>Preferred equity - Blixt</t>
-        </is>
+      <c r="B297" s="306">
+        <f>"Preferred equity - "&amp;Cover!$B$10</f>
+        <v/>
       </c>
       <c r="H297" s="1062">
         <f>+H312</f>
@@ -47694,10 +47690,9 @@
     </row>
     <row r="308" ht="15" customHeight="1">
       <c r="A308" s="307" t="n"/>
-      <c r="B308" s="3" t="inlineStr">
-        <is>
-          <t>Preferred equity - Blixt</t>
-        </is>
+      <c r="B308" s="3">
+        <f>"Preferred equity - "&amp;Cover!$B$10</f>
+        <v/>
       </c>
       <c r="C308" s="18" t="n"/>
       <c r="D308" s="18" t="n"/>
@@ -47779,10 +47774,9 @@
         <v/>
       </c>
       <c r="O310" s="1062" t="n"/>
-      <c r="P310" s="1136" t="inlineStr">
-        <is>
-          <t>Assumes 100% of new funding is provided by Blixt, i.e. no pre-emption from other shareholders</t>
-        </is>
+      <c r="P310" s="1136">
+        <f>"Assumes 100% of new funding is provided by "&amp;Cover!$B$10&amp;", i.e. no pre-emption from other shareholders"</f>
+        <v/>
       </c>
     </row>
     <row r="311" ht="15" customHeight="1">
@@ -49407,10 +49401,9 @@
     </row>
     <row r="361" ht="15" customFormat="1" customHeight="1" s="21">
       <c r="A361" s="459" t="n"/>
-      <c r="B361" s="90" t="inlineStr">
-        <is>
-          <t>Less Blixt Exit Fee</t>
-        </is>
+      <c r="B361" s="90">
+        <f>"Less "&amp;Cover!$B$10&amp;" Exit Fee"</f>
+        <v/>
       </c>
       <c r="C361" s="7" t="n"/>
       <c r="D361" s="7" t="n"/>
@@ -49491,10 +49484,9 @@
     </row>
     <row r="363" ht="15" customFormat="1" customHeight="1" s="21">
       <c r="A363" s="459" t="n"/>
-      <c r="B363" s="90" t="inlineStr">
-        <is>
-          <t>Less: Blixt prefs</t>
-        </is>
+      <c r="B363" s="90">
+        <f>"Less: "&amp;Cover!$B$10&amp;" prefs"</f>
+        <v/>
       </c>
       <c r="C363" s="7" t="n"/>
       <c r="D363" s="7" t="n"/>
@@ -50059,10 +50051,9 @@
     </row>
     <row r="379" ht="15" customHeight="1">
       <c r="A379" s="307" t="n"/>
-      <c r="B379" s="18" t="inlineStr">
-        <is>
-          <t>Blixt returns</t>
-        </is>
+      <c r="B379" s="18">
+        <f>Cover!$B$10&amp;" returns"</f>
+        <v/>
       </c>
       <c r="C379" s="18" t="n"/>
       <c r="D379" s="18" t="n"/>
@@ -50080,10 +50071,9 @@
     </row>
     <row r="380" ht="15" customHeight="1">
       <c r="A380" s="307" t="n"/>
-      <c r="B380" s="1" t="inlineStr">
-        <is>
-          <t>Blixt entry equity value</t>
-        </is>
+      <c r="B380" s="1">
+        <f>Cover!$B$10&amp;" entry equity value"</f>
+        <v/>
       </c>
       <c r="I380" s="1206">
         <f>+$E$102</f>
@@ -50113,10 +50103,9 @@
     </row>
     <row r="381" ht="15" customHeight="1">
       <c r="A381" s="307" t="n"/>
-      <c r="B381" s="1" t="inlineStr">
-        <is>
-          <t>Blixt equity injection</t>
-        </is>
+      <c r="B381" s="1">
+        <f>Cover!$B$10&amp;" equity injection"</f>
+        <v/>
       </c>
       <c r="I381" s="1206">
         <f>+I231</f>
@@ -50146,10 +50135,9 @@
     </row>
     <row r="382" ht="15" customHeight="1">
       <c r="A382" s="307" t="n"/>
-      <c r="B382" s="308" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Blixt equity </t>
-        </is>
+      <c r="B382" s="308">
+        <f>"Total "&amp;Cover!$B$10&amp;" equity "</f>
+        <v/>
       </c>
       <c r="C382" s="308" t="n"/>
       <c r="D382" s="308" t="n"/>
@@ -51507,10 +51495,9 @@
           <t>x</t>
         </is>
       </c>
-      <c r="B424" s="106" t="inlineStr">
-        <is>
-          <t>Blixt Returns</t>
-        </is>
+      <c r="B424" s="106">
+        <f>Cover!$B$10&amp;" Returns"</f>
+        <v/>
       </c>
       <c r="C424" s="106" t="n"/>
       <c r="D424" s="106" t="n"/>
@@ -55202,10 +55189,9 @@
       <c r="P550" s="1292" t="n"/>
     </row>
     <row r="551" ht="15" customHeight="1">
-      <c r="B551" s="9" t="inlineStr">
-        <is>
-          <t>Total Blixt equity invested / EBITDA</t>
-        </is>
+      <c r="B551" s="9">
+        <f>"Total "&amp;Cover!$B$10&amp;" equity invested / EBITDA"</f>
+        <v/>
       </c>
       <c r="C551" s="40" t="n"/>
       <c r="D551" s="40" t="n"/>
@@ -55728,7 +55714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:S82"/>
+  <dimension ref="A1:S82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23.5703125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -55738,6 +55724,7 @@
     <col width="13.85546875" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="790" t="n">
         <v>1</v>
@@ -55762,6 +55749,7 @@
       <c r="P2" s="849" t="n"/>
       <c r="Q2" s="849" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="C4" s="789" t="inlineStr">
         <is>
@@ -55786,6 +55774,7 @@
       <c r="P4" s="789" t="n"/>
       <c r="Q4" s="683" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="C6" s="813" t="inlineStr">
         <is>
@@ -56285,10 +56274,9 @@
         <f>I14/I10</f>
         <v/>
       </c>
-      <c r="K15" s="833" t="inlineStr">
-        <is>
-          <t>Blixt returned Equity</t>
-        </is>
+      <c r="K15" s="833">
+        <f>Cover!$B$10&amp;" returned Equity"</f>
+        <v/>
       </c>
       <c r="L15" s="833" t="n"/>
       <c r="M15" s="826" t="n"/>
@@ -56472,10 +56460,9 @@
         <f>I18/I10</f>
         <v/>
       </c>
-      <c r="K19" s="823" t="inlineStr">
-        <is>
-          <t>Blixt exposure</t>
-        </is>
+      <c r="K19" s="823">
+        <f>Cover!$B$10&amp;" exposure"</f>
+        <v/>
       </c>
       <c r="L19" s="1355">
         <f>LBO!J382</f>
@@ -56506,10 +56493,9 @@
       <c r="G20" s="830" t="n"/>
       <c r="H20" s="830" t="n"/>
       <c r="I20" s="830" t="n"/>
-      <c r="K20" s="825" t="inlineStr">
-        <is>
-          <t>Blixt returns</t>
-        </is>
+      <c r="K20" s="825">
+        <f>Cover!$B$10&amp;" returns"</f>
+        <v/>
       </c>
       <c r="L20" s="1363" t="n"/>
       <c r="M20" s="1363" t="n"/>
@@ -56976,6 +56962,7 @@
         <v/>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="B36" s="790" t="n">
         <v>2</v>
@@ -57000,6 +56987,8 @@
       <c r="P36" s="849" t="n"/>
       <c r="Q36" s="849" t="n"/>
     </row>
+    <row r="37"/>
+    <row r="38"/>
     <row r="39" ht="23.25" customHeight="1">
       <c r="C39" s="873" t="n"/>
       <c r="D39" s="873" t="n"/>
@@ -57141,10 +57130,9 @@
       <c r="J43" s="883" t="n"/>
     </row>
     <row r="44" ht="23.25" customHeight="1">
-      <c r="C44" s="877" t="inlineStr">
-        <is>
-          <t>Blixt returns (£m)</t>
-        </is>
+      <c r="C44" s="877">
+        <f>Cover!$B$10&amp;" returns (£m)"</f>
+        <v/>
       </c>
       <c r="D44" s="873" t="n"/>
       <c r="E44" s="874" t="inlineStr">
@@ -57294,6 +57282,7 @@
         <v/>
       </c>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="B50" s="790" t="n">
         <v>3</v>
@@ -57318,6 +57307,8 @@
       <c r="P50" s="849" t="n"/>
       <c r="Q50" s="849" t="n"/>
     </row>
+    <row r="51"/>
+    <row r="52"/>
     <row r="53" ht="30" customHeight="1">
       <c r="D53" s="814" t="inlineStr">
         <is>
@@ -58450,6 +58441,8 @@
       <c r="H79" s="852" t="n"/>
       <c r="S79" s="768" t="n"/>
     </row>
+    <row r="80"/>
+    <row r="81"/>
     <row r="82">
       <c r="C82" t="inlineStr">
         <is>
@@ -58499,7 +58492,7 @@
     <col width="9.140625" customWidth="1" min="29" max="31"/>
     <col width="17.85546875" bestFit="1" customWidth="1" min="32" max="32"/>
     <col width="9.140625" customWidth="1" min="33" max="40"/>
-    <col hidden="1" min="41" max="48"/>
+    <col hidden="1" width="13" customWidth="1" min="41" max="48"/>
     <col hidden="1" width="9.140625" customWidth="1" style="175" min="49" max="16384"/>
   </cols>
   <sheetData>
@@ -60520,10 +60513,9 @@
     </row>
     <row r="28" ht="12.75" customFormat="1" customHeight="1" s="196">
       <c r="B28" s="1384" t="n"/>
-      <c r="C28" s="231" t="inlineStr">
-        <is>
-          <t>Blixt management fee</t>
-        </is>
+      <c r="C28" s="231">
+        <f>Cover!$B$10&amp;" management fee"</f>
+        <v/>
       </c>
       <c r="D28" s="205" t="n"/>
       <c r="E28" s="353" t="n"/>
@@ -60928,10 +60920,9 @@
     </row>
     <row r="35" ht="12.75" customFormat="1" customHeight="1" s="196">
       <c r="B35" s="1384" t="n"/>
-      <c r="C35" s="231" t="inlineStr">
-        <is>
-          <t>Blixt equity injection</t>
-        </is>
+      <c r="C35" s="231">
+        <f>Cover!$B$10&amp;" equity injection"</f>
+        <v/>
       </c>
       <c r="D35" s="240" t="n"/>
       <c r="E35" s="353" t="n"/>
@@ -61206,10 +61197,9 @@
         <v/>
       </c>
       <c r="O40" s="204" t="n"/>
-      <c r="P40" s="523" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Memo: Blixt day 1 cheque </t>
-        </is>
+      <c r="P40" s="523">
+        <f>"Memo: "&amp;Cover!$B$10&amp;" day 1 cheque "</f>
+        <v/>
       </c>
       <c r="R40" s="1446">
         <f>+R24+R26+R32</f>
@@ -61632,10 +61622,9 @@
         <f>+IFERROR(G46/((+I16/H16-1)*100),"n/a")</f>
         <v/>
       </c>
-      <c r="H49" s="242" t="inlineStr">
-        <is>
-          <t>Less Blixt exit fees</t>
-        </is>
+      <c r="H49" s="242">
+        <f>"Less "&amp;Cover!$B$10&amp;" exit fees"</f>
+        <v/>
       </c>
       <c r="I49" s="203" t="n"/>
       <c r="J49" s="1464" t="n"/>
@@ -61750,10 +61739,9 @@
     </row>
     <row r="52" ht="12.75" customFormat="1" customHeight="1" s="196">
       <c r="B52" s="1384" t="n"/>
-      <c r="C52" s="210" t="inlineStr">
-        <is>
-          <t>Total Blixt equity / EBITDA</t>
-        </is>
+      <c r="C52" s="210">
+        <f>"Total "&amp;Cover!$B$10&amp;" equity / EBITDA"</f>
+        <v/>
       </c>
       <c r="D52" s="202" t="n"/>
       <c r="E52" s="1468">
@@ -61768,10 +61756,9 @@
         <f>IFERROR((+LBO!G83+LBO!D91+LBO!D85+LBO!G98)/I16,"n/a")</f>
         <v/>
       </c>
-      <c r="H52" s="242" t="inlineStr">
-        <is>
-          <t>Blixt Ords and prefs</t>
-        </is>
+      <c r="H52" s="242">
+        <f>Cover!$B$10&amp;" Ords and prefs"</f>
+        <v/>
       </c>
       <c r="I52" s="203" t="n"/>
       <c r="J52" s="1433" t="n"/>
@@ -61936,10 +61923,9 @@
     </row>
     <row r="56" ht="12.75" customFormat="1" customHeight="1" s="196">
       <c r="B56" s="1384" t="n"/>
-      <c r="C56" s="242" t="inlineStr">
-        <is>
-          <t>Day 1 Blixt equity / EBITDA</t>
-        </is>
+      <c r="C56" s="242">
+        <f>"Day 1 "&amp;Cover!$B$10&amp;" equity / EBITDA"</f>
+        <v/>
       </c>
       <c r="D56" s="202" t="n"/>
       <c r="E56" s="1468">
@@ -61954,10 +61940,9 @@
         <f>IFERROR((+LBO!$E$83+LBO!$E$91+LBO!$E$85)/I16,"n/a")</f>
         <v/>
       </c>
-      <c r="H56" s="210" t="inlineStr">
-        <is>
-          <t>Blixt entry equity + injections</t>
-        </is>
+      <c r="H56" s="210">
+        <f>Cover!$B$10&amp;" entry equity + injections"</f>
+        <v/>
       </c>
       <c r="I56" s="202" t="n"/>
       <c r="J56" s="202" t="n"/>
@@ -61998,10 +61983,9 @@
       <c r="E57" s="1457" t="n"/>
       <c r="F57" s="1457" t="n"/>
       <c r="G57" s="1470" t="n"/>
-      <c r="H57" s="298" t="inlineStr">
-        <is>
-          <t>Blixt Capital Gain</t>
-        </is>
+      <c r="H57" s="298">
+        <f>Cover!$B$10&amp;" Capital Gain"</f>
+        <v/>
       </c>
       <c r="I57" s="295" t="n"/>
       <c r="J57" s="295" t="n"/>
@@ -62042,10 +62026,9 @@
       <c r="E58" s="1475" t="n"/>
       <c r="F58" s="1475" t="n"/>
       <c r="G58" s="1476" t="n"/>
-      <c r="H58" s="512" t="inlineStr">
-        <is>
-          <t>Blixt CoC (x)</t>
-        </is>
+      <c r="H58" s="512">
+        <f>Cover!$B$10&amp;" CoC (x)"</f>
+        <v/>
       </c>
       <c r="I58" s="513" t="n"/>
       <c r="J58" s="513" t="n"/>
@@ -63433,7 +63416,7 @@
       <c r="AU155" s="175" t="n"/>
       <c r="AV155" s="175" t="n"/>
     </row>
-    <row r="156" hidden="1" customHeight="1">
+    <row r="156" hidden="1">
       <c r="AB156" s="175" t="n"/>
       <c r="AC156" s="175" t="n"/>
       <c r="AD156" s="175" t="n"/>
@@ -63456,7 +63439,7 @@
       <c r="AU156" s="175" t="n"/>
       <c r="AV156" s="175" t="n"/>
     </row>
-    <row r="157" hidden="1" customHeight="1">
+    <row r="157" hidden="1">
       <c r="AB157" s="175" t="n"/>
       <c r="AC157" s="175" t="n"/>
       <c r="AD157" s="175" t="n"/>
@@ -63479,7 +63462,7 @@
       <c r="AU157" s="175" t="n"/>
       <c r="AV157" s="175" t="n"/>
     </row>
-    <row r="158" hidden="1" customHeight="1">
+    <row r="158" hidden="1">
       <c r="AB158" s="175" t="n"/>
       <c r="AC158" s="175" t="n"/>
       <c r="AD158" s="175" t="n"/>
@@ -63502,7 +63485,7 @@
       <c r="AU158" s="175" t="n"/>
       <c r="AV158" s="175" t="n"/>
     </row>
-    <row r="159" hidden="1" customHeight="1">
+    <row r="159" hidden="1">
       <c r="AB159" s="175" t="n"/>
       <c r="AC159" s="175" t="n"/>
       <c r="AD159" s="175" t="n"/>
@@ -63525,7 +63508,7 @@
       <c r="AU159" s="175" t="n"/>
       <c r="AV159" s="175" t="n"/>
     </row>
-    <row r="160" hidden="1" customHeight="1">
+    <row r="160" hidden="1">
       <c r="AB160" s="175" t="n"/>
       <c r="AC160" s="175" t="n"/>
       <c r="AD160" s="175" t="n"/>
@@ -63548,7 +63531,7 @@
       <c r="AU160" s="175" t="n"/>
       <c r="AV160" s="175" t="n"/>
     </row>
-    <row r="161" hidden="1" customFormat="1" customHeight="1" s="175"/>
+    <row r="161" hidden="1" customFormat="1" s="175"/>
   </sheetData>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2362204724409449" right="0.3543307086614174" top="0.1574803149606299" bottom="0.1574803149606299" header="0.1574803149606299" footer="0.1574803149606299"/>
@@ -63571,12 +63554,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="683" t="inlineStr">
         <is>
@@ -63711,7 +63695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:X95"/>
+  <dimension ref="A1:X95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.85546875" customWidth="1" min="2" max="2"/>
@@ -63722,6 +63706,7 @@
     <col width="15.7109375" customWidth="1" min="19" max="21"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="788" t="n">
         <v>1</v>
@@ -63750,6 +63735,7 @@
       <c r="T2" s="789" t="n"/>
       <c r="U2" s="789" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="E4" s="790" t="inlineStr">
         <is>
@@ -63779,6 +63765,7 @@
       <c r="F5" s="1495" t="n"/>
       <c r="G5" s="1495" t="n"/>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="B7" s="788" t="n">
         <v>2</v>
@@ -63807,6 +63794,7 @@
       <c r="T7" s="789" t="n"/>
       <c r="U7" s="789" t="n"/>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="D9" s="801" t="inlineStr">
         <is>
@@ -65238,6 +65226,7 @@
       <c r="S40" s="789" t="n"/>
       <c r="T40" s="789" t="n"/>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="D42" s="788" t="inlineStr">
         <is>
@@ -65286,6 +65275,7 @@
         <v/>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="C44" s="683" t="inlineStr">
         <is>
@@ -66715,6 +66705,7 @@
         <v/>
       </c>
     </row>
+    <row r="78"/>
     <row r="79">
       <c r="B79" s="788" t="n">
         <v>5</v>
@@ -66742,6 +66733,7 @@
       <c r="S79" s="789" t="n"/>
       <c r="T79" s="789" t="n"/>
     </row>
+    <row r="80"/>
     <row r="81">
       <c r="E81" s="798" t="n">
         <v>46357</v>
@@ -66780,6 +66772,8 @@
         <v>-1.1</v>
       </c>
     </row>
+    <row r="83"/>
+    <row r="84"/>
     <row r="85">
       <c r="B85" s="788" t="n">
         <v>6</v>
@@ -66807,6 +66801,8 @@
       <c r="S85" s="789" t="n"/>
       <c r="T85" s="789" t="n"/>
     </row>
+    <row r="86"/>
+    <row r="87"/>
     <row r="88">
       <c r="C88" t="inlineStr">
         <is>
@@ -66828,6 +66824,8 @@
         <v/>
       </c>
     </row>
+    <row r="90"/>
+    <row r="91"/>
     <row r="92">
       <c r="E92" s="683" t="inlineStr">
         <is>

</xml_diff>